<commit_message>
WIP: Rename all intervals
</commit_message>
<xml_diff>
--- a/_documentation/Intervals.xlsx
+++ b/_documentation/Intervals.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="17766"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\philippe.matray\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repo\midiminuit\_documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12296"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -374,9 +374,6 @@
     <t>diminished octave</t>
   </si>
   <si>
-    <t>Chromatic semitone, minor semitone</t>
-  </si>
-  <si>
     <t>A1</t>
   </si>
   <si>
@@ -518,9 +515,6 @@
     <t>925 or 947</t>
   </si>
   <si>
-    <t>Diminished eighth</t>
-  </si>
-  <si>
     <t>d8</t>
   </si>
   <si>
@@ -567,6 +561,12 @@
   </si>
   <si>
     <t>A4, TT</t>
+  </si>
+  <si>
+    <t>chromatic semitone, minor semitone</t>
+  </si>
+  <si>
+    <t>diminished eighth</t>
   </si>
 </sst>
 </file>
@@ -636,9 +636,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -646,9 +643,12 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -928,38 +928,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.4140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.25" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.4140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.4140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.4140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.58203125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="D1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="6"/>
+      <c r="F1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2" t="s">
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
@@ -988,14 +988,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>68</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1010,7 +1010,7 @@
       <c r="G3" s="1">
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I3" s="1">
@@ -1023,14 +1023,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>39</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -1045,7 +1045,7 @@
       <c r="G4" s="1">
         <v>5</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>33</v>
       </c>
       <c r="I4" s="1">
@@ -1058,14 +1058,14 @@
         <v>498</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>39</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>70</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -1078,7 +1078,7 @@
         <v>7</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>30</v>
@@ -1093,17 +1093,17 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>39</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="1" t="s">
@@ -1128,18 +1128,18 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>40</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>72</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>50</v>
@@ -1163,17 +1163,17 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>40</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -1198,17 +1198,17 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>40</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>74</v>
       </c>
       <c r="E9" s="1" t="s">
@@ -1233,14 +1233,14 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>40</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>82</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -1268,18 +1268,18 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>92</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>91</v>
@@ -1288,17 +1288,17 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>41</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -1323,14 +1323,14 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>41</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>98</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -1358,17 +1358,17 @@
         <v>104</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>41</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E14" s="1" t="s">
@@ -1393,21 +1393,21 @@
         <v>112</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>42</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>86</v>
@@ -1416,33 +1416,33 @@
         <v>86</v>
       </c>
       <c r="H15" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="K15" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>122</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>77</v>
@@ -1451,7 +1451,7 @@
         <v>77</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>96</v>
@@ -1460,20 +1460,20 @@
         <v>96</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>42</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D17" s="5" t="s">
+      <c r="C17" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E17" s="1" t="s">
@@ -1485,7 +1485,7 @@
       <c r="G17" s="1">
         <v>5</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="H17" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I17" s="1">
@@ -1498,56 +1498,56 @@
         <v>457</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>42</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="F18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G18" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>42</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>101</v>
@@ -1556,7 +1556,7 @@
         <v>59</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>103</v>
@@ -1565,24 +1565,24 @@
         <v>103</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>137</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>109</v>
@@ -1591,7 +1591,7 @@
         <v>51</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>111</v>
@@ -1600,24 +1600,24 @@
         <v>111</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>42</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>141</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>35</v>
@@ -1626,7 +1626,7 @@
         <v>36</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>38</v>
@@ -1635,56 +1635,56 @@
         <v>89</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>42</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C22" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D22" s="5" t="s">
+      <c r="F22" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>173</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>86</v>
       </c>
       <c r="H22" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="K22" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="I22" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>43</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>145</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>36</v>
@@ -1693,33 +1693,33 @@
         <v>36</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>36</v>
       </c>
       <c r="J23" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="K23" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="K23" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>43</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>51</v>
@@ -1728,7 +1728,7 @@
         <v>51</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>53</v>
@@ -1737,24 +1737,24 @@
         <v>53</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>43</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>155</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>59</v>
@@ -1763,7 +1763,7 @@
         <v>59</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>61</v>
@@ -1772,55 +1772,55 @@
         <v>61</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>43</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="F26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G26" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="K26" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>43</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="1" t="s">
@@ -1832,7 +1832,7 @@
       <c r="G27" s="1">
         <v>5</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H27" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I27" s="1">
@@ -1845,21 +1845,21 @@
         <v>743</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>43</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>76</v>
@@ -1868,7 +1868,7 @@
         <v>77</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>79</v>
@@ -1877,24 +1877,24 @@
         <v>79</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>43</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="3" t="s">
         <v>113</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>85</v>
@@ -1903,7 +1903,7 @@
         <v>86</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>88</v>
@@ -1912,43 +1912,43 @@
         <v>88</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>44</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>44</v>
       </c>

</xml_diff>

<commit_message>
Add inverse intervals and interval classes
</commit_message>
<xml_diff>
--- a/_documentation/Intervals.xlsx
+++ b/_documentation/Intervals.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="17766"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repo\midiminuit\_documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12296"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="175">
   <si>
     <t>Diminished sixth</t>
   </si>
@@ -530,27 +531,6 @@
     <t>5</t>
   </si>
   <si>
-    <t>Augmented octave</t>
-  </si>
-  <si>
-    <t>Augmented eighth</t>
-  </si>
-  <si>
-    <t>A8</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>25:12</t>
-  </si>
-  <si>
-    <t>1300</t>
-  </si>
-  <si>
-    <t>1271</t>
-  </si>
-  <si>
     <t>semitone, half tone, half step</t>
   </si>
   <si>
@@ -567,13 +547,16 @@
   </si>
   <si>
     <t>diminished eighth</t>
+  </si>
+  <si>
+    <t>=MOD(B1,6)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -585,6 +568,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -632,7 +623,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -646,9 +637,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -927,23 +919,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.4140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.58203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.4140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.4140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.4140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.58203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="88.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D1" s="6" t="s">
         <v>5</v>
       </c>
@@ -959,7 +951,7 @@
       <c r="J1" s="6"/>
       <c r="K1" s="6"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
@@ -988,11 +980,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C3" s="5" t="s">
@@ -1023,11 +1015,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="7" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="5" t="s">
@@ -1058,11 +1050,11 @@
         <v>498</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="7" t="s">
         <v>24</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -1093,11 +1085,11 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1128,18 +1120,18 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="7" t="s">
         <v>45</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>72</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>50</v>
@@ -1163,11 +1155,11 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="7" t="s">
         <v>55</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -1198,11 +1190,11 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="7" t="s">
         <v>64</v>
       </c>
       <c r="C9" s="5" t="s">
@@ -1233,11 +1225,11 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="7" t="s">
         <v>81</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -1268,18 +1260,18 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>92</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>91</v>
@@ -1287,12 +1279,15 @@
       <c r="F11" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G11" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -1323,11 +1318,11 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="7" t="s">
         <v>56</v>
       </c>
       <c r="C13" s="5" t="s">
@@ -1358,11 +1353,11 @@
         <v>104</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="7" t="s">
         <v>49</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -1393,18 +1388,18 @@
         <v>112</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="7" t="s">
         <v>113</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>116</v>
@@ -1428,11 +1423,11 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="7" t="s">
         <v>47</v>
       </c>
       <c r="C16" s="5" t="s">
@@ -1463,11 +1458,11 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -1498,11 +1493,11 @@
         <v>457</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="7" t="s">
         <v>157</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -1512,7 +1507,7 @@
         <v>125</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>126</v>
@@ -1533,11 +1528,11 @@
         <v>129</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="7" t="s">
         <v>130</v>
       </c>
       <c r="C19" s="5" t="s">
@@ -1568,11 +1563,11 @@
         <v>134</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C20" s="5" t="s">
@@ -1603,11 +1598,11 @@
         <v>138</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="7" t="s">
         <v>105</v>
       </c>
       <c r="C21" s="3" t="s">
@@ -1638,318 +1633,286 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>168</v>
+        <v>43</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>48</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>169</v>
+        <v>57</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>170</v>
+        <v>144</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>171</v>
+        <v>36</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>86</v>
+        <v>36</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>173</v>
+        <v>36</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>48</v>
+      <c r="B23" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>146</v>
+        <v>53</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>93</v>
+      <c r="B24" s="7" t="s">
+        <v>152</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>57</v>
+      <c r="B25" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>125</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>59</v>
+        <v>126</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>59</v>
+        <v>126</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>61</v>
+        <v>128</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>61</v>
+        <v>128</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>125</v>
+      <c r="B26" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>57</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>4</v>
+      </c>
+      <c r="F26" s="1">
+        <v>7</v>
+      </c>
+      <c r="G26" s="1">
+        <v>5</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="1">
+        <v>700</v>
+      </c>
+      <c r="J26" s="1">
+        <v>700</v>
+      </c>
+      <c r="K26" s="1">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>0</v>
+      <c r="B27" s="7" t="s">
+        <v>106</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>15</v>
+        <v>159</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F27" s="1">
-        <v>7</v>
-      </c>
-      <c r="G27" s="1">
-        <v>5</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" s="1">
-        <v>700</v>
-      </c>
-      <c r="J27" s="1">
-        <v>700</v>
-      </c>
-      <c r="K27" s="1">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>160</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>106</v>
+      <c r="B28" s="7" t="s">
+        <v>114</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>57</v>
+        <v>113</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>43</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1978,15 +1941,391 @@
     <hyperlink ref="C19" r:id="rId16" tooltip="Diminished fourth" display="https://en.wikipedia.org/wiki/Diminished_fourth"/>
     <hyperlink ref="C20" r:id="rId17" tooltip="Diminished third" display="https://en.wikipedia.org/wiki/Diminished_third"/>
     <hyperlink ref="C21" r:id="rId18" tooltip="Diminished second" display="https://en.wikipedia.org/wiki/Diminished_second"/>
-    <hyperlink ref="C23" r:id="rId19" tooltip="Augmented seventh" display="https://en.wikipedia.org/wiki/Augmented_seventh"/>
-    <hyperlink ref="C24" r:id="rId20" tooltip="Augmented sixth" display="https://en.wikipedia.org/wiki/Augmented_sixth"/>
-    <hyperlink ref="C25" r:id="rId21" tooltip="Augmented fifth" display="https://en.wikipedia.org/wiki/Augmented_fifth"/>
-    <hyperlink ref="C27" r:id="rId22" tooltip="Augmented third" display="https://en.wikipedia.org/wiki/Augmented_third"/>
-    <hyperlink ref="C28" r:id="rId23" tooltip="Augmented second" display="https://en.wikipedia.org/wiki/Augmented_second"/>
-    <hyperlink ref="C29" r:id="rId24" tooltip="Augmented unison" display="https://en.wikipedia.org/wiki/Augmented_unison"/>
-    <hyperlink ref="C22" r:id="rId25" location="Diminished_unison" tooltip="Augmented unison" display="https://en.wikipedia.org/wiki/Augmented_unison - Diminished_unison"/>
+    <hyperlink ref="C22" r:id="rId19" tooltip="Augmented seventh" display="https://en.wikipedia.org/wiki/Augmented_seventh"/>
+    <hyperlink ref="C23" r:id="rId20" tooltip="Augmented sixth" display="https://en.wikipedia.org/wiki/Augmented_sixth"/>
+    <hyperlink ref="C24" r:id="rId21" tooltip="Augmented fifth" display="https://en.wikipedia.org/wiki/Augmented_fifth"/>
+    <hyperlink ref="C26" r:id="rId22" tooltip="Augmented third" display="https://en.wikipedia.org/wiki/Augmented_third"/>
+    <hyperlink ref="C27" r:id="rId23" tooltip="Augmented second" display="https://en.wikipedia.org/wiki/Augmented_second"/>
+    <hyperlink ref="C28" r:id="rId24" tooltip="Augmented unison" display="https://en.wikipedia.org/wiki/Augmented_unison"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId26"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId25"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="1">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="1">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="1">
+        <v>5</v>
+      </c>
+      <c r="C15" s="1">
+        <v>5</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="1">
+        <v>7</v>
+      </c>
+      <c r="C24" s="1">
+        <v>5</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>